<commit_message>
Another intermediate commit before everything goes to shit
</commit_message>
<xml_diff>
--- a/OSB_Gilder/test_chamber/TEST_singular_9.xlsx
+++ b/OSB_Gilder/test_chamber/TEST_singular_9.xlsx
@@ -2444,7 +2444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T1045"/>
+  <dimension ref="A1:T1049"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5078125" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8.77" customWidth="1" style="63" min="1" max="1"/>
@@ -2453,19 +2453,17 @@
     <col width="8.880000000000001" customWidth="1" style="63" min="4" max="4"/>
     <col width="4.78" customWidth="1" style="63" min="5" max="5"/>
     <col width="10.78" customWidth="1" style="63" min="6" max="6"/>
-    <col width="2.77" customWidth="1" style="63" min="7" max="7"/>
-    <col width="74.77" customWidth="1" style="63" min="8" max="8"/>
-    <col width="4" customWidth="1" style="63" min="9" max="9"/>
-    <col width="50" customWidth="1" style="63" min="10" max="10"/>
-    <col width="13" customWidth="1" style="63" min="11" max="12"/>
-    <col width="10" customWidth="1" style="56" min="12" max="12"/>
-    <col width="10" customWidth="1" style="63" min="13" max="13"/>
+    <col width="4" customWidth="1" style="63" min="7" max="7"/>
+    <col width="50" customWidth="1" style="63" min="8" max="8"/>
+    <col width="13" customWidth="1" style="63" min="9" max="9"/>
+    <col width="10" customWidth="1" style="63" min="10" max="10"/>
+    <col width="10" customWidth="1" style="63" min="11" max="12"/>
+    <col width="15" customWidth="1" style="56" min="12" max="12"/>
+    <col width="15" customWidth="1" style="63" min="13" max="13"/>
     <col width="15" customWidth="1" style="63" min="14" max="19"/>
-    <col width="15" customWidth="1" style="56" min="15" max="15"/>
-    <col width="15" customWidth="1" style="56" min="16" max="16"/>
+    <col width="50" customWidth="1" style="56" min="15" max="15"/>
+    <col width="50" customWidth="1" style="56" min="16" max="16"/>
     <col width="50" customWidth="1" style="56" min="17" max="17"/>
-    <col width="50" customWidth="1" style="56" min="18" max="18"/>
-    <col width="50" customWidth="1" style="56" min="19" max="19"/>
     <col width="169.33" customWidth="1" style="63" min="20" max="20"/>
   </cols>
   <sheetData>
@@ -55698,71 +55696,81 @@
       <c r="T1022" s="90" t="n"/>
     </row>
     <row r="1023">
+      <c r="G1023" s="136" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="H1023" s="136" t="inlineStr">
+        <is>
+          <t>NAME</t>
+        </is>
+      </c>
       <c r="I1023" s="136" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Debit_Total</t>
         </is>
       </c>
       <c r="J1023" s="136" t="inlineStr">
         <is>
-          <t>NAME</t>
+          <t>Debit_NC</t>
         </is>
       </c>
       <c r="K1023" s="136" t="inlineStr">
         <is>
-          <t>Debit_Total</t>
+          <t>Debit_IC</t>
         </is>
       </c>
       <c r="L1023" s="136" t="inlineStr">
         <is>
-          <t>Debit_NC</t>
+          <t>Credit_Total</t>
         </is>
       </c>
       <c r="M1023" s="136" t="inlineStr">
         <is>
-          <t>Debit_IC</t>
+          <t>Credit_NC</t>
         </is>
       </c>
       <c r="N1023" s="136" t="inlineStr">
         <is>
-          <t>Credit_Total</t>
+          <t>Credit_IC</t>
         </is>
       </c>
       <c r="O1023" s="136" t="inlineStr">
         <is>
-          <t>Credit_NC</t>
+          <t>Balance_Total</t>
         </is>
       </c>
       <c r="P1023" s="136" t="inlineStr">
         <is>
-          <t>Credit_IC</t>
+          <t>Balance_NC</t>
         </is>
       </c>
       <c r="Q1023" s="136" t="inlineStr">
         <is>
-          <t>Balance_Total</t>
-        </is>
-      </c>
-      <c r="R1023" s="136" t="inlineStr">
-        <is>
-          <t>Balance_NC</t>
-        </is>
-      </c>
-      <c r="S1023" s="136" t="inlineStr">
-        <is>
           <t>Balance_IC</t>
         </is>
       </c>
     </row>
     <row r="1024">
-      <c r="I1024" s="137" t="n">
+      <c r="G1024" s="137" t="n">
         <v>1</v>
       </c>
-      <c r="J1024" s="137" t="inlineStr">
+      <c r="H1024" s="137" t="inlineStr">
         <is>
           <t>Проценти по ОВДП (коди 6120-6122)</t>
         </is>
       </c>
+      <c r="I1024" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J1024" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="K1024" s="138" t="inlineStr">
         <is>
           <t>-</t>
@@ -55783,38 +55791,38 @@
           <t>-</t>
         </is>
       </c>
-      <c r="O1024" s="138" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P1024" s="138" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q1024" s="138">
+      <c r="O1024" s="138">
         <f>Q599 + SUM(Q600:Q601) + SUM(Q602:Q603)</f>
         <v/>
       </c>
-      <c r="R1024" s="138">
+      <c r="P1024" s="138">
         <f>R599 + SUM(R600:R601) + SUM(R602:R603)</f>
         <v/>
       </c>
-      <c r="S1024" s="138">
+      <c r="Q1024" s="138">
         <f>S599 + SUM(S600:S601) + SUM(S602:S603)</f>
         <v/>
       </c>
     </row>
     <row r="1025">
-      <c r="I1025" s="137" t="n">
+      <c r="G1025" s="137" t="n">
         <v>2</v>
       </c>
-      <c r="J1025" s="137" t="inlineStr">
+      <c r="H1025" s="137" t="inlineStr">
         <is>
           <t>Проценти по ДС (коди 6127-6128)</t>
         </is>
       </c>
+      <c r="I1025" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J1025" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="K1025" s="138" t="inlineStr">
         <is>
           <t>-</t>
@@ -55835,38 +55843,38 @@
           <t>-</t>
         </is>
       </c>
-      <c r="O1025" s="138" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P1025" s="138" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q1025" s="138">
+      <c r="O1025" s="138">
         <f>SUM(Q609:Q610) + SUM(Q611:Q612)</f>
         <v/>
       </c>
-      <c r="R1025" s="138">
+      <c r="P1025" s="138">
         <f>SUM(R609:R610) + SUM(R611:R612)</f>
         <v/>
       </c>
-      <c r="S1025" s="138">
+      <c r="Q1025" s="138">
         <f>SUM(S609:S610) + SUM(S611:S612)</f>
         <v/>
       </c>
     </row>
     <row r="1026">
-      <c r="I1026" s="137" t="n">
+      <c r="G1026" s="137" t="n">
         <v>3</v>
       </c>
-      <c r="J1026" s="137" t="inlineStr">
+      <c r="H1026" s="137" t="inlineStr">
         <is>
           <t>Обсяг ДС (код 1430, 1440)</t>
         </is>
       </c>
+      <c r="I1026" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J1026" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="K1026" s="138" t="inlineStr">
         <is>
           <t>-</t>
@@ -55887,142 +55895,142 @@
           <t>-</t>
         </is>
       </c>
-      <c r="O1026" s="138" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P1026" s="138" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q1026" s="138">
+      <c r="O1026" s="138">
         <f>Q52 + Q57</f>
         <v/>
       </c>
-      <c r="R1026" s="138">
+      <c r="P1026" s="138">
         <f>R52 + R57</f>
         <v/>
       </c>
-      <c r="S1026" s="138">
+      <c r="Q1026" s="138">
         <f>S52 + S57</f>
         <v/>
       </c>
     </row>
     <row r="1027">
-      <c r="I1027" s="137" t="n">
+      <c r="G1027" s="137" t="n">
         <v>4</v>
       </c>
-      <c r="J1027" s="137" t="inlineStr">
+      <c r="H1027" s="137" t="inlineStr">
         <is>
           <t>Кошти в НБУ (кор.рахунок) (кредит) (код 1200)</t>
         </is>
       </c>
+      <c r="I1027" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J1027" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="K1027" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1027" s="138" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M1027" s="138" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N1027" s="138">
+      <c r="L1027" s="138">
         <f>M26</f>
         <v/>
       </c>
-      <c r="O1027" s="138">
+      <c r="M1027" s="138">
         <f>O26</f>
         <v/>
       </c>
-      <c r="P1027" s="138">
+      <c r="N1027" s="138">
         <f>P26</f>
         <v/>
       </c>
+      <c r="O1027" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P1027" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="Q1027" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="R1027" s="138" t="inlineStr">
+    </row>
+    <row r="1028">
+      <c r="G1028" s="137" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1028" s="137" t="inlineStr">
+        <is>
+          <t>Кошти в НБУ (УСЬОГО) (кредит) (розділ 12)</t>
+        </is>
+      </c>
+      <c r="I1028" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="S1027" s="138" t="inlineStr">
+      <c r="J1028" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-    </row>
-    <row r="1028">
-      <c r="I1028" s="137" t="n">
-        <v>5</v>
-      </c>
-      <c r="J1028" s="137" t="inlineStr">
-        <is>
-          <t>Кошти в НБУ (УСЬОГО) (кредит) (розділ 12)</t>
-        </is>
-      </c>
       <c r="K1028" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1028" s="138" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M1028" s="138" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N1028" s="138">
+      <c r="L1028" s="138">
         <f>SUM(M26:M29)</f>
         <v/>
       </c>
-      <c r="O1028" s="138">
+      <c r="M1028" s="138">
         <f>SUM(O26:O29)</f>
         <v/>
       </c>
-      <c r="P1028" s="138">
+      <c r="N1028" s="138">
         <f>SUM(P26:P29)</f>
         <v/>
       </c>
+      <c r="O1028" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P1028" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="Q1028" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="R1028" s="138" t="inlineStr">
+    </row>
+    <row r="1029">
+      <c r="G1029" s="137" t="n">
+        <v>6</v>
+      </c>
+      <c r="H1029" s="137" t="inlineStr">
+        <is>
+          <t>Процентні доходи (коди р.60,р.61)</t>
+        </is>
+      </c>
+      <c r="I1029" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="S1028" s="138" t="inlineStr">
+      <c r="J1029" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-    </row>
-    <row r="1029">
-      <c r="I1029" s="137" t="n">
-        <v>6</v>
-      </c>
-      <c r="J1029" s="137" t="inlineStr">
-        <is>
-          <t>Процентні доходи (коди р.60,р.61)</t>
-        </is>
-      </c>
       <c r="K1029" s="138" t="inlineStr">
         <is>
           <t>-</t>
@@ -56043,857 +56051,1055 @@
           <t>-</t>
         </is>
       </c>
-      <c r="O1029" s="138" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P1029" s="138" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q1029" s="138">
+      <c r="O1029" s="138">
         <f>SUM(Q531:Q532, Q534:Q545, Q547:Q562, Q564:Q569, Q571:Q574, Q576:Q583, Q585:Q590, Q592:Q593) + SUM(Q596:Q597, Q599:Q612, Q614:Q615)</f>
         <v/>
       </c>
-      <c r="R1029" s="138">
+      <c r="P1029" s="138">
         <f>SUM(R531:R532, R534:R545, R547:R562, R564:R569, R571:R574, R576:R583, R585:R590, R592:R593) + SUM(R596:R597, R599:R612, R614:R615)</f>
         <v/>
       </c>
-      <c r="S1029" s="138">
+      <c r="Q1029" s="138">
         <f>SUM(S531:S532, S534:S545, S547:S562, S564:S569, S571:S574, S576:S583, S585:S590, S592:S593) + SUM(S596:S597, S599:S612, S614:S615)</f>
         <v/>
       </c>
     </row>
     <row r="1030">
-      <c r="I1030" s="137" t="n">
+      <c r="G1030" s="137" t="n">
         <v>7</v>
       </c>
-      <c r="J1030" s="137" t="inlineStr">
+      <c r="H1030" s="137" t="inlineStr">
+        <is>
+          <t>Проценти по ДС у % до процентних доходів</t>
+        </is>
+      </c>
+      <c r="I1030" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J1030" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K1030" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L1030" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M1030" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N1030" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O1030" s="138">
+        <f>(O1025 / O1029) * 100</f>
+        <v/>
+      </c>
+      <c r="P1030" s="138">
+        <f>(P1025 / P1029) * 100</f>
+        <v/>
+      </c>
+      <c r="Q1030" s="138">
+        <f>(Q1025 / Q1029) * 100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="G1031" s="137" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1031" s="137" t="inlineStr">
+        <is>
+          <t>Проценти по ОВДП у % до процентних доходів</t>
+        </is>
+      </c>
+      <c r="I1031" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J1031" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K1031" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L1031" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M1031" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N1031" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O1031" s="138">
+        <f>(O1024 / O1029) * 100</f>
+        <v/>
+      </c>
+      <c r="P1031" s="138">
+        <f>(P1024 / P1029) * 100</f>
+        <v/>
+      </c>
+      <c r="Q1031" s="138">
+        <f>(Q1024 / Q1029) * 100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="G1032" s="137" t="n">
+        <v>9</v>
+      </c>
+      <c r="H1032" s="137" t="inlineStr">
+        <is>
+          <t>Проценти по ДС+ОВДП у % до процентних доходів</t>
+        </is>
+      </c>
+      <c r="I1032" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J1032" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K1032" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L1032" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M1032" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N1032" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O1032" s="138">
+        <f>O1030 + O1031</f>
+        <v/>
+      </c>
+      <c r="P1032" s="138">
+        <f>P1030 + P1031</f>
+        <v/>
+      </c>
+      <c r="Q1032" s="138">
+        <f>Q1030 + Q1031</f>
+        <v/>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="G1033" s="137" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1033" s="137" t="inlineStr">
         <is>
           <t>Проценти за кредитами НК (коди 602, 603, 609)</t>
         </is>
       </c>
-      <c r="K1030" s="138" t="inlineStr">
+      <c r="I1033" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1030" s="138" t="inlineStr">
+      <c r="J1033" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M1030" s="138" t="inlineStr">
+      <c r="K1033" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N1030" s="138" t="inlineStr">
+      <c r="L1033" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O1030" s="138" t="inlineStr">
+      <c r="M1033" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P1030" s="138" t="inlineStr">
+      <c r="N1033" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q1030" s="138">
+      <c r="O1033" s="138">
         <f>SUM(Q547:Q562) + SUM(Q564:Q569) + SUM(Q592:Q593)</f>
         <v/>
       </c>
-      <c r="R1030" s="138">
+      <c r="P1033" s="138">
         <f>SUM(R547:R562) + SUM(R564:R569) + SUM(R592:R593)</f>
         <v/>
       </c>
-      <c r="S1030" s="138">
+      <c r="Q1033" s="138">
         <f>SUM(S547:S562) + SUM(S564:S569) + SUM(S592:S593)</f>
         <v/>
       </c>
     </row>
-    <row r="1031">
-      <c r="I1031" s="137" t="n">
-        <v>8</v>
-      </c>
-      <c r="J1031" s="137" t="inlineStr">
+    <row r="1034">
+      <c r="G1034" s="137" t="n">
+        <v>11</v>
+      </c>
+      <c r="H1034" s="137" t="inlineStr">
         <is>
           <t>Проценти за кредитами ДГ (коди 605, 606, 611)</t>
         </is>
       </c>
-      <c r="K1031" s="138" t="inlineStr">
+      <c r="I1034" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1031" s="138" t="inlineStr">
+      <c r="J1034" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M1031" s="138" t="inlineStr">
+      <c r="K1034" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N1031" s="138" t="inlineStr">
+      <c r="L1034" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O1031" s="138" t="inlineStr">
+      <c r="M1034" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P1031" s="138" t="inlineStr">
+      <c r="N1034" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q1031" s="138">
+      <c r="O1034" s="138">
         <f>SUM(Q576:Q583) + SUM(Q585:Q590) + SUM(Q596:Q597)</f>
         <v/>
       </c>
-      <c r="R1031" s="138">
+      <c r="P1034" s="138">
         <f>SUM(R576:R583) + SUM(R585:R590) + SUM(R596:R597)</f>
         <v/>
       </c>
-      <c r="S1031" s="138">
+      <c r="Q1034" s="138">
         <f>SUM(S576:S583) + SUM(S585:S590) + SUM(S596:S597)</f>
         <v/>
       </c>
     </row>
-    <row r="1032">
-      <c r="I1032" s="137" t="n">
-        <v>9</v>
-      </c>
-      <c r="J1032" s="137" t="inlineStr">
+    <row r="1035">
+      <c r="G1035" s="137" t="n">
+        <v>12</v>
+      </c>
+      <c r="H1035" s="137" t="inlineStr">
         <is>
           <t>Проценти за кредитами ЗДУ (код 604)</t>
         </is>
       </c>
-      <c r="K1032" s="138" t="inlineStr">
+      <c r="I1035" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1032" s="138" t="inlineStr">
+      <c r="J1035" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M1032" s="138" t="inlineStr">
+      <c r="K1035" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N1032" s="138" t="inlineStr">
+      <c r="L1035" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O1032" s="138" t="inlineStr">
+      <c r="M1035" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P1032" s="138" t="inlineStr">
+      <c r="N1035" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q1032" s="138">
+      <c r="O1035" s="138">
         <f>SUM(Q571:Q574)</f>
         <v/>
       </c>
-      <c r="R1032" s="138">
+      <c r="P1035" s="138">
         <f>SUM(R571:R574)</f>
         <v/>
       </c>
-      <c r="S1032" s="138">
+      <c r="Q1035" s="138">
         <f>SUM(S571:S574)</f>
         <v/>
       </c>
     </row>
-    <row r="1033">
-      <c r="I1033" s="137" t="n">
-        <v>10</v>
-      </c>
-      <c r="J1033" s="137" t="inlineStr">
+    <row r="1036">
+      <c r="G1036" s="137" t="n">
+        <v>13</v>
+      </c>
+      <c r="H1036" s="137" t="inlineStr">
         <is>
           <t>Проценти за поточними вкладами ДГ (код 7040)</t>
         </is>
       </c>
-      <c r="K1033" s="138" t="inlineStr">
+      <c r="I1036" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1033" s="138" t="inlineStr">
+      <c r="J1036" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M1033" s="138" t="inlineStr">
+      <c r="K1036" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N1033" s="138" t="inlineStr">
+      <c r="L1036" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O1033" s="138" t="inlineStr">
+      <c r="M1036" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P1033" s="138" t="inlineStr">
+      <c r="N1036" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q1033" s="138">
+      <c r="O1036" s="138">
         <f>SUM(Q720:Q721)</f>
         <v/>
       </c>
-      <c r="R1033" s="138">
+      <c r="P1036" s="138">
         <f>SUM(R720:R721)</f>
         <v/>
       </c>
-      <c r="S1033" s="138">
+      <c r="Q1036" s="138">
         <f>SUM(S720:S721)</f>
         <v/>
       </c>
     </row>
-    <row r="1034">
-      <c r="I1034" s="137" t="n">
-        <v>11</v>
-      </c>
-      <c r="J1034" s="137" t="inlineStr">
+    <row r="1037">
+      <c r="G1037" s="137" t="n">
+        <v>14</v>
+      </c>
+      <c r="H1037" s="137" t="inlineStr">
         <is>
           <t>Проценти за строковими вкладами ДГ (код 7041)</t>
         </is>
       </c>
-      <c r="K1034" s="138" t="inlineStr">
+      <c r="I1037" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1034" s="138" t="inlineStr">
+      <c r="J1037" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M1034" s="138" t="inlineStr">
+      <c r="K1037" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N1034" s="138" t="inlineStr">
+      <c r="L1037" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O1034" s="138" t="inlineStr">
+      <c r="M1037" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P1034" s="138" t="inlineStr">
+      <c r="N1037" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q1034" s="138">
+      <c r="O1037" s="138">
         <f>SUM(Q722:Q723)</f>
         <v/>
       </c>
-      <c r="R1034" s="138">
+      <c r="P1037" s="138">
         <f>SUM(R722:R723)</f>
         <v/>
       </c>
-      <c r="S1034" s="138">
+      <c r="Q1037" s="138">
         <f>SUM(S722:S723)</f>
         <v/>
       </c>
     </row>
-    <row r="1035">
-      <c r="I1035" s="137" t="n">
-        <v>12</v>
-      </c>
-      <c r="J1035" s="137" t="inlineStr">
+    <row r="1038">
+      <c r="G1038" s="137" t="n">
+        <v>15</v>
+      </c>
+      <c r="H1038" s="137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Процентні витрати банків ДГ - всього </t>
+        </is>
+      </c>
+      <c r="I1038" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J1038" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K1038" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L1038" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M1038" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N1038" s="138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O1038" s="138">
+        <f>O1036 + O1037</f>
+        <v/>
+      </c>
+      <c r="P1038" s="138">
+        <f>P1036 + P1037</f>
+        <v/>
+      </c>
+      <c r="Q1038" s="138">
+        <f>Q1036 + Q1037</f>
+        <v/>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="G1039" s="137" t="n">
+        <v>16</v>
+      </c>
+      <c r="H1039" s="137" t="inlineStr">
         <is>
           <t>Кредити субʼєктам господарювання (р.20, р.23, 260)</t>
         </is>
       </c>
-      <c r="K1035" s="138" t="inlineStr">
+      <c r="I1039" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1035" s="138" t="inlineStr">
+      <c r="J1039" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M1035" s="138" t="inlineStr">
+      <c r="K1039" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N1035" s="138" t="inlineStr">
+      <c r="L1039" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O1035" s="138" t="inlineStr">
+      <c r="M1039" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P1035" s="138" t="inlineStr">
+      <c r="N1039" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q1035" s="138">
+      <c r="O1039" s="138">
         <f>SUM(Q88:Q126) + SUM(Q167:Q176) + SUM(Q186:Q188)</f>
         <v/>
       </c>
-      <c r="R1035" s="138">
+      <c r="P1039" s="138">
         <f>SUM(R88:R126) + SUM(R167:R176) + SUM(R186:R188)</f>
         <v/>
       </c>
-      <c r="S1035" s="138">
+      <c r="Q1039" s="138">
         <f>SUM(S88:S126) + SUM(S167:S176) + SUM(S186:S188)</f>
         <v/>
       </c>
     </row>
-    <row r="1036">
-      <c r="I1036" s="137" t="n">
-        <v>13</v>
-      </c>
-      <c r="J1036" s="137" t="inlineStr">
+    <row r="1040">
+      <c r="G1040" s="137" t="n">
+        <v>17</v>
+      </c>
+      <c r="H1040" s="137" t="inlineStr">
         <is>
           <t>Кредити ЗДУ (р.21)</t>
         </is>
       </c>
-      <c r="K1036" s="138" t="inlineStr">
+      <c r="I1040" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1036" s="138" t="inlineStr">
+      <c r="J1040" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M1036" s="138" t="inlineStr">
+      <c r="K1040" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N1036" s="138" t="inlineStr">
+      <c r="L1040" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O1036" s="138" t="inlineStr">
+      <c r="M1040" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P1036" s="138" t="inlineStr">
+      <c r="N1040" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q1036" s="138">
+      <c r="O1040" s="138">
         <f>SUM(Q128:Q141)</f>
         <v/>
       </c>
-      <c r="R1036" s="138">
+      <c r="P1040" s="138">
         <f>SUM(R128:R141)</f>
         <v/>
       </c>
-      <c r="S1036" s="138">
+      <c r="Q1040" s="138">
         <f>SUM(S128:S141)</f>
         <v/>
       </c>
     </row>
-    <row r="1037">
-      <c r="I1037" s="137" t="n">
-        <v>14</v>
-      </c>
-      <c r="J1037" s="137" t="inlineStr">
+    <row r="1041">
+      <c r="G1041" s="137" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1041" s="137" t="inlineStr">
         <is>
           <t>Кредити фізичним особам (р. 22, 24, 262)</t>
         </is>
       </c>
-      <c r="K1037" s="138" t="inlineStr">
+      <c r="I1041" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1037" s="138" t="inlineStr">
+      <c r="J1041" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M1037" s="138" t="inlineStr">
+      <c r="K1041" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N1037" s="138" t="inlineStr">
+      <c r="L1041" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O1037" s="138" t="inlineStr">
+      <c r="M1041" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P1037" s="138" t="inlineStr">
+      <c r="N1041" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q1037" s="138">
+      <c r="O1041" s="138">
         <f>SUM(Q143:Q165) + SUM(Q178:Q184) + SUM(Q189:Q192)</f>
         <v/>
       </c>
-      <c r="R1037" s="138">
+      <c r="P1041" s="138">
         <f>SUM(R143:R165) + SUM(R178:R184) + SUM(R189:R192)</f>
         <v/>
       </c>
-      <c r="S1037" s="138">
+      <c r="Q1041" s="138">
         <f>SUM(S143:S165) + SUM(S178:S184) + SUM(S189:S192)</f>
         <v/>
       </c>
     </row>
-    <row r="1038">
-      <c r="I1038" s="137" t="n">
-        <v>15</v>
-      </c>
-      <c r="J1038" s="137" t="inlineStr">
+    <row r="1042">
+      <c r="G1042" s="137" t="n">
+        <v>19</v>
+      </c>
+      <c r="H1042" s="137" t="inlineStr">
         <is>
           <t>Кредити небанківським установам (265)</t>
         </is>
       </c>
-      <c r="K1038" s="138" t="inlineStr">
+      <c r="I1042" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1038" s="138" t="inlineStr">
+      <c r="J1042" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M1038" s="138" t="inlineStr">
+      <c r="K1042" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N1038" s="138" t="inlineStr">
+      <c r="L1042" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O1038" s="138" t="inlineStr">
+      <c r="M1042" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P1038" s="138" t="inlineStr">
+      <c r="N1042" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q1038" s="138">
+      <c r="O1042" s="138">
         <f>SUM(Q193:Q195)</f>
         <v/>
       </c>
-      <c r="R1038" s="138">
+      <c r="P1042" s="138">
         <f>SUM(R193:R195)</f>
         <v/>
       </c>
-      <c r="S1038" s="138">
+      <c r="Q1042" s="138">
         <f>SUM(S193:S195)</f>
         <v/>
       </c>
     </row>
-    <row r="1039">
-      <c r="I1039" s="137" t="n">
-        <v>16</v>
-      </c>
-      <c r="J1039" s="137" t="inlineStr">
+    <row r="1043">
+      <c r="G1043" s="137" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1043" s="137" t="inlineStr">
         <is>
           <t>Прибуток звітного року (5040)</t>
         </is>
       </c>
-      <c r="K1039" s="138" t="inlineStr">
+      <c r="I1043" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1039" s="138" t="inlineStr">
+      <c r="J1043" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M1039" s="138" t="inlineStr">
+      <c r="K1043" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N1039" s="138" t="inlineStr">
+      <c r="L1043" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O1039" s="138" t="inlineStr">
+      <c r="M1043" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P1039" s="138" t="inlineStr">
+      <c r="N1043" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q1039" s="138">
+      <c r="O1043" s="138">
         <f>Q509</f>
         <v/>
       </c>
-      <c r="R1039" s="138">
+      <c r="P1043" s="138">
         <f>R509</f>
         <v/>
       </c>
-      <c r="S1039" s="138">
+      <c r="Q1043" s="138">
         <f>S509</f>
         <v/>
       </c>
     </row>
-    <row r="1040">
-      <c r="I1040" s="137" t="n">
-        <v>17</v>
-      </c>
-      <c r="J1040" s="137" t="inlineStr">
+    <row r="1044">
+      <c r="G1044" s="137" t="n">
+        <v>21</v>
+      </c>
+      <c r="H1044" s="137" t="inlineStr">
         <is>
           <t>Збиток звітного року (5041)</t>
         </is>
       </c>
-      <c r="K1040" s="138" t="inlineStr">
+      <c r="I1044" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1040" s="138" t="inlineStr">
+      <c r="J1044" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M1040" s="138" t="inlineStr">
+      <c r="K1044" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N1040" s="138" t="inlineStr">
+      <c r="L1044" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O1040" s="138" t="inlineStr">
+      <c r="M1044" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P1040" s="138" t="inlineStr">
+      <c r="N1044" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q1040" s="138">
+      <c r="O1044" s="138">
         <f>Q510</f>
         <v/>
       </c>
-      <c r="R1040" s="138">
+      <c r="P1044" s="138">
         <f>R510</f>
         <v/>
       </c>
-      <c r="S1040" s="138">
+      <c r="Q1044" s="138">
         <f>S510</f>
         <v/>
       </c>
     </row>
-    <row r="1041">
-      <c r="I1041" s="137" t="n">
-        <v>18</v>
-      </c>
-      <c r="J1041" s="137" t="inlineStr">
+    <row r="1045">
+      <c r="G1045" s="137" t="n">
+        <v>22</v>
+      </c>
+      <c r="H1045" s="137" t="inlineStr">
         <is>
           <t>Податок на прибуток (7900)</t>
         </is>
       </c>
-      <c r="K1041" s="138" t="inlineStr">
+      <c r="I1045" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1041" s="138" t="inlineStr">
+      <c r="J1045" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M1041" s="138" t="inlineStr">
+      <c r="K1045" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N1041" s="138" t="inlineStr">
+      <c r="L1045" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O1041" s="138" t="inlineStr">
+      <c r="M1045" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P1041" s="138" t="inlineStr">
+      <c r="N1045" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q1041" s="138">
+      <c r="O1045" s="138">
         <f>SUM(Q831:Q832)</f>
         <v/>
       </c>
-      <c r="R1041" s="138">
+      <c r="P1045" s="138">
         <f>SUM(R831:R832)</f>
         <v/>
       </c>
-      <c r="S1041" s="138">
+      <c r="Q1045" s="138">
         <f>SUM(S831:S832)</f>
         <v/>
       </c>
     </row>
-    <row r="1042">
-      <c r="I1042" s="137" t="n">
-        <v>19</v>
-      </c>
-      <c r="J1042" s="137" t="inlineStr">
+    <row r="1046">
+      <c r="G1046" s="137" t="n">
+        <v>23</v>
+      </c>
+      <c r="H1046" s="137" t="inlineStr">
         <is>
           <t>Інші податки (741)</t>
         </is>
       </c>
-      <c r="K1042" s="138" t="inlineStr">
+      <c r="I1046" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1042" s="138" t="inlineStr">
+      <c r="J1046" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M1042" s="138" t="inlineStr">
+      <c r="K1046" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N1042" s="138" t="inlineStr">
+      <c r="L1046" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O1042" s="138" t="inlineStr">
+      <c r="M1046" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P1042" s="138" t="inlineStr">
+      <c r="N1046" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q1042" s="138">
+      <c r="O1046" s="138">
         <f>SUM(Q775:Q778)</f>
         <v/>
       </c>
-      <c r="R1042" s="138">
+      <c r="P1046" s="138">
         <f>SUM(R775:R778)</f>
         <v/>
       </c>
-      <c r="S1042" s="138">
+      <c r="Q1046" s="138">
         <f>SUM(S775:S778)</f>
         <v/>
       </c>
     </row>
-    <row r="1043">
-      <c r="I1043" s="137" t="n">
-        <v>20</v>
-      </c>
-      <c r="J1043" s="137" t="inlineStr">
+    <row r="1047">
+      <c r="G1047" s="137" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1047" s="137" t="inlineStr">
         <is>
           <t>Відрахування в резерви (770)</t>
         </is>
       </c>
-      <c r="K1043" s="138" t="inlineStr">
+      <c r="I1047" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1043" s="138" t="inlineStr">
+      <c r="J1047" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M1043" s="138" t="inlineStr">
+      <c r="K1047" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N1043" s="138" t="inlineStr">
+      <c r="L1047" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O1043" s="138" t="inlineStr">
+      <c r="M1047" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P1043" s="138" t="inlineStr">
+      <c r="N1047" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q1043" s="138">
+      <c r="O1047" s="138">
         <f>SUM(Q813:Q828)</f>
         <v/>
       </c>
-      <c r="R1043" s="138">
+      <c r="P1047" s="138">
         <f>SUM(R813:R828)</f>
         <v/>
       </c>
-      <c r="S1043" s="138">
+      <c r="Q1047" s="138">
         <f>SUM(S813:S828)</f>
         <v/>
       </c>
     </row>
-    <row r="1044">
-      <c r="I1044" s="137" t="n">
-        <v>21</v>
-      </c>
-      <c r="J1044" s="137" t="inlineStr">
+    <row r="1048">
+      <c r="G1048" s="137" t="n">
+        <v>25</v>
+      </c>
+      <c r="H1048" s="137" t="inlineStr">
         <is>
           <t>Загальні доходи (6)</t>
         </is>
       </c>
-      <c r="K1044" s="138" t="inlineStr">
+      <c r="I1048" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1044" s="138" t="inlineStr">
+      <c r="J1048" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M1044" s="138" t="inlineStr">
+      <c r="K1048" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N1044" s="138" t="inlineStr">
+      <c r="L1048" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O1044" s="138" t="inlineStr">
+      <c r="M1048" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P1044" s="138" t="inlineStr">
+      <c r="N1048" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q1044" s="138">
+      <c r="O1048" s="138">
         <f>SUM(Q531:Q532, Q534:Q545, Q547:Q562, Q564:Q569, Q571:Q574, Q576:Q583, Q585:Q590, Q592:Q593, Q596:Q597, Q599:Q612, Q614:Q615, Q618:Q626, Q628:Q635, Q637:Q642, Q645:Q647, Q649, Q651, Q653, Q655, Q657, Q659:Q667, Q670:Q671, Q674:Q678, Q680:Q686, Q688, Q691:Q694)</f>
         <v/>
       </c>
-      <c r="R1044" s="138">
+      <c r="P1048" s="138">
         <f>SUM(R531:R532, R534:R545, R547:R562, R564:R569, R571:R574, R576:R583, R585:R590, R592:R593, R596:R597, R599:R612, R614:R615, R618:R626, R628:R635, R637:R642, R645:R647, R649, R651, R653, R655, R657, R659:R667, R670:R671, R674:R678, R680:R686, R688, R691:R694)</f>
         <v/>
       </c>
-      <c r="S1044" s="138">
+      <c r="Q1048" s="138">
         <f>SUM(S531:S532, S534:S545, S547:S562, S564:S569, S571:S574, S576:S583, S585:S590, S592:S593, S596:S597, S599:S612, S614:S615, S618:S626, S628:S635, S637:S642, S645:S647, S649, S651, S653, S655, S657, S659:S667, S670:S671, S674:S678, S680:S686, S688, S691:S694)</f>
         <v/>
       </c>
     </row>
-    <row r="1045">
-      <c r="I1045" s="137" t="n">
-        <v>22</v>
-      </c>
-      <c r="J1045" s="137" t="inlineStr">
+    <row r="1049">
+      <c r="G1049" s="137" t="n">
+        <v>26</v>
+      </c>
+      <c r="H1049" s="137" t="inlineStr">
         <is>
           <t>Загальні витрати (7)</t>
         </is>
       </c>
-      <c r="K1045" s="138" t="inlineStr">
+      <c r="I1049" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L1045" s="138" t="inlineStr">
+      <c r="J1049" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M1045" s="138" t="inlineStr">
+      <c r="K1049" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N1045" s="138" t="inlineStr">
+      <c r="L1049" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O1045" s="138" t="inlineStr">
+      <c r="M1049" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P1045" s="138" t="inlineStr">
+      <c r="N1049" s="138" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q1045" s="138">
+      <c r="O1049" s="138">
         <f>SUM(Q701, Q703:Q709, Q711:Q716, Q718, Q720:Q725, Q727:Q728, Q730:Q732, Q735:Q736, Q738:Q741, Q744:Q745, Q747, Q749, Q751, Q753, Q755, Q757:Q765, Q768:Q773, Q775:Q778, Q780:Q783, Q785:Q788, Q790:Q795, Q797:Q800, Q803:Q808, Q810, Q813:Q828, Q831:Q832)</f>
         <v/>
       </c>
-      <c r="R1045" s="138">
+      <c r="P1049" s="138">
         <f>SUM(R701, R703:R709, R711:R716, R718, R720:R725, R727:R728, R730:R732, R735:R736, R738:R741, R744:R745, R747, R749, R751, R753, R755, R757:R765, R768:R773, R775:R778, R780:R783, R785:R788, R790:R795, R797:R800, R803:R808, R810, R813:R828, R831:R832)</f>
         <v/>
       </c>
-      <c r="S1045" s="138">
+      <c r="Q1049" s="138">
         <f>SUM(S701, S703:S709, S711:S716, S718, S720:S725, S727:S728, S730:S732, S735:S736, S738:S741, S744:S745, S747, S749, S751, S753, S755, S757:S765, S768:S773, S775:S778, S780:S783, S785:S788, S790:S795, S797:S800, S803:S808, S810, S813:S828, S831:S832)</f>
         <v/>
       </c>

</xml_diff>